<commit_message>
Add classifier fixes: loss curve, combined metrics plot, train split eval
- Add ANN epoch-error (loss) curve plot
- Add grouped bar chart of all 6 metrics on one figure
- Evaluate all models on training split in addition to val/test
- Add loop comments per coding standard #4
- Bump version to v1.1
</commit_message>
<xml_diff>
--- a/code/output/model_performance.xlsx
+++ b/code/output/model_performance.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,26 +466,26 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>validation</t>
+          <t>train</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.9642982149107455</v>
+        <v>0.9686328105468425</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9642057697100578</v>
+        <v>0.9685293221817567</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9642982149107455</v>
+        <v>0.9686328105468425</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9768902907221636</v>
+        <v>0.9798280278222845</v>
       </c>
       <c r="G2" t="n">
-        <v>0.964023713019734</v>
+        <v>0.968427932918792</v>
       </c>
       <c r="H2" t="n">
-        <v>0.9907678308321465</v>
+        <v>0.9928389881302613</v>
       </c>
     </row>
     <row r="3">
@@ -496,56 +496,56 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>test</t>
+          <t>validation</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.9699530046995301</v>
+        <v>0.9642982149107455</v>
       </c>
       <c r="D3" t="n">
-        <v>0.969864496493862</v>
+        <v>0.9642057697100578</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9699530046995301</v>
+        <v>0.9642982149107455</v>
       </c>
       <c r="F3" t="n">
-        <v>0.9805563546239338</v>
+        <v>0.9768902907221636</v>
       </c>
       <c r="G3" t="n">
-        <v>0.9697464795300955</v>
+        <v>0.964023713019734</v>
       </c>
       <c r="H3" t="n">
-        <v>0.9924789254821275</v>
+        <v>0.9907678308321465</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Decision Tree</t>
+          <t>ANN</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>validation</t>
+          <t>test</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.9210960548027401</v>
+        <v>0.9699530046995301</v>
       </c>
       <c r="D4" t="n">
-        <v>0.9209601993065444</v>
+        <v>0.969864496493862</v>
       </c>
       <c r="E4" t="n">
-        <v>0.9210960548027401</v>
+        <v>0.9699530046995301</v>
       </c>
       <c r="F4" t="n">
-        <v>0.9503503886603584</v>
+        <v>0.9805563546239338</v>
       </c>
       <c r="G4" t="n">
-        <v>0.9210057055929792</v>
+        <v>0.9697464795300955</v>
       </c>
       <c r="H4" t="n">
-        <v>0.9255255829905378</v>
+        <v>0.9924789254821275</v>
       </c>
     </row>
     <row r="5">
@@ -556,32 +556,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>test</t>
+          <t>train</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.9215578442155784</v>
+        <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>0.9215707056614443</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>0.9215578442155784</v>
+        <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>0.950929980133783</v>
+        <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>0.9215434069502429</v>
+        <v>1</v>
       </c>
       <c r="H5" t="n">
-        <v>0.9263949702006744</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>K-NN</t>
+          <t>Decision Tree</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -590,28 +590,28 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.9224461223061153</v>
+        <v>0.9210960548027401</v>
       </c>
       <c r="D6" t="n">
-        <v>0.9236741757414144</v>
+        <v>0.9209601993065444</v>
       </c>
       <c r="E6" t="n">
-        <v>0.9224461223061153</v>
+        <v>0.9210960548027401</v>
       </c>
       <c r="F6" t="n">
-        <v>0.9473719405092819</v>
+        <v>0.9503503886603584</v>
       </c>
       <c r="G6" t="n">
-        <v>0.9218125115615665</v>
+        <v>0.9210057055929792</v>
       </c>
       <c r="H6" t="n">
-        <v>0.9619007051067705</v>
+        <v>0.9255255829905378</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>K-NN</t>
+          <t>Decision Tree</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -620,81 +620,201 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.9277572242775722</v>
+        <v>0.9215578442155784</v>
       </c>
       <c r="D7" t="n">
-        <v>0.9289323960925385</v>
+        <v>0.9215707056614443</v>
       </c>
       <c r="E7" t="n">
-        <v>0.9277572242775722</v>
+        <v>0.9215578442155784</v>
       </c>
       <c r="F7" t="n">
-        <v>0.950797950169247</v>
+        <v>0.950929980133783</v>
       </c>
       <c r="G7" t="n">
-        <v>0.9272344324563389</v>
+        <v>0.9215434069502429</v>
       </c>
       <c r="H7" t="n">
-        <v>0.9661538195465608</v>
+        <v>0.9263949702006744</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SVM</t>
+          <t>K-NN</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>validation</t>
+          <t>train</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.9488474423721186</v>
+        <v>0.937282288038134</v>
       </c>
       <c r="D8" t="n">
-        <v>0.9487195954844315</v>
+        <v>0.9382426734615221</v>
       </c>
       <c r="E8" t="n">
-        <v>0.9488474423721186</v>
+        <v>0.937282288038134</v>
       </c>
       <c r="F8" t="n">
-        <v>0.9655833291570998</v>
+        <v>0.9573418549568928</v>
       </c>
       <c r="G8" t="n">
-        <v>0.9480658948683208</v>
+        <v>0.9367091114849593</v>
       </c>
       <c r="H8" t="n">
-        <v>0.979140769120023</v>
+        <v>0.9893474404393636</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>K-NN</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>validation</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0.9224461223061153</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.9236741757414144</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.9224461223061153</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.9473719405092819</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.9218125115615665</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.9619007051067705</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>K-NN</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0.9277572242775722</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.9289323960925385</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.9277572242775722</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.950797950169247</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.9272344324563389</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.9661538195465608</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>SVM</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>train</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0.9525158752645877</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.9523531950337825</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.9525158752645877</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.967949318787508</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.9518445399400774</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.9820233042175897</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>SVM</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>validation</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0.9488474423721186</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.9487195954844315</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.9488474423721186</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.9655833291570998</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.9480658948683208</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.979140769120023</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>SVM</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
         <is>
           <t>test</t>
         </is>
       </c>
-      <c r="C9" t="n">
+      <c r="C13" t="n">
         <v>0.9547045295470453</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D13" t="n">
         <v>0.954654060168205</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E13" t="n">
         <v>0.9547045295470453</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F13" t="n">
         <v>0.9693121484525511</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G13" t="n">
         <v>0.9541081708018527</v>
       </c>
-      <c r="H9" t="n">
+      <c r="H13" t="n">
         <v>0.9820562537105441</v>
       </c>
     </row>

</xml_diff>